<commit_message>
Update physiology analysis to approved 85-subject cohort
</commit_message>
<xml_diff>
--- a/supplementary/Supplementary_Physiology_Cohort_and_Trial_Counts.xlsx
+++ b/supplementary/Supplementary_Physiology_Cohort_and_Trial_Counts.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R75a3d37581e24e8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Included Subjects" sheetId="2" r:id="R12b7a743620a480c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Subjects" sheetId="3" r:id="R346a546dd1ba4115"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIR and Protocol" sheetId="4" r:id="Rfc5521257d4d45dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8bf2040337b5436c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Included Subjects" sheetId="2" r:id="R0815fa0e0c484542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Subjects" sheetId="3" r:id="R08cde9ebc31e49aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FIR and Protocol" sheetId="4" r:id="Rfa6a196c626648f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -68,7 +68,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF7E6"/>
+        <x:fgColor rgb="FFEAF0F7"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -368,7 +368,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>EEG Motor Movement Imagery Database physiology cohort used in the manuscript</x:v>
+        <x:v>Updated 85-subject cohort based on the documented 300 microvolt rejection criterion</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -399,10 +399,10 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="11" t="str">
-        <x:v>Manuscript physiology cohort</x:v>
+        <x:v>Updated physiology cohort</x:v>
       </x:c>
       <x:c r="B7" s="11" t="n">
-        <x:v>76</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -410,7 +410,7 @@
         <x:v>Subjects outside physiology cohort</x:v>
       </x:c>
       <x:c r="B8" s="11" t="n">
-        <x:v>27</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -421,14 +421,7 @@
         <x:v>18</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
-      <x:c r="A10" s="11" t="str">
-        <x:v>Archived cohort exclusions without an additional recorded criterion</x:v>
-      </x:c>
-      <x:c r="B10" s="11" t="n">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
+    <x:row r="10"/>
     <x:row r="11"/>
     <x:row r="12" ht="48" hidden="0" customHeight="1">
       <x:c r="A12" s="9" t="str">
@@ -458,22 +451,22 @@
         <x:v>Rest</x:v>
       </x:c>
       <x:c r="B13" s="11" t="n">
-        <x:v>5097</x:v>
+        <x:v>5225</x:v>
       </x:c>
       <x:c r="C13" s="12" t="n">
-        <x:v>67.0657894736842</x:v>
+        <x:v>61.470588235294116</x:v>
       </x:c>
       <x:c r="D13" s="11" t="n">
-        <x:v>86</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="E13" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F13" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="G13" s="11" t="n">
-        <x:v>76</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -481,10 +474,10 @@
         <x:v>Left fist imagery</x:v>
       </x:c>
       <x:c r="B14" s="11" t="n">
-        <x:v>1404</x:v>
+        <x:v>1448</x:v>
       </x:c>
       <x:c r="C14" s="12" t="n">
-        <x:v>18.473684210526315</x:v>
+        <x:v>17.03529411764706</x:v>
       </x:c>
       <x:c r="D14" s="11" t="n">
         <x:v>21</x:v>
@@ -496,7 +489,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="G14" s="11" t="n">
-        <x:v>76</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -504,10 +497,10 @@
         <x:v>Right fist imagery</x:v>
       </x:c>
       <x:c r="B15" s="11" t="n">
-        <x:v>1385</x:v>
+        <x:v>1436</x:v>
       </x:c>
       <x:c r="C15" s="12" t="n">
-        <x:v>18.223684210526315</x:v>
+        <x:v>16.894117647058824</x:v>
       </x:c>
       <x:c r="D15" s="11" t="n">
         <x:v>21</x:v>
@@ -519,7 +512,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="G15" s="11" t="n">
-        <x:v>76</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
@@ -527,10 +520,10 @@
         <x:v>Both feet imagery</x:v>
       </x:c>
       <x:c r="B16" s="11" t="n">
-        <x:v>1401</x:v>
+        <x:v>1460</x:v>
       </x:c>
       <x:c r="C16" s="12" t="n">
-        <x:v>18.43421052631579</x:v>
+        <x:v>17.176470588235293</x:v>
       </x:c>
       <x:c r="D16" s="11" t="n">
         <x:v>21</x:v>
@@ -542,7 +535,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="G16" s="11" t="n">
-        <x:v>76</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="17"/>
@@ -567,7 +560,7 @@
         <x:v>Unequal retained counts across all four classes</x:v>
       </x:c>
       <x:c r="B20" s="11" t="n">
-        <x:v>76</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
@@ -601,24 +594,12 @@
       <x:c r="F24" s="16"/>
       <x:c r="G24" s="16"/>
     </x:row>
-    <x:row r="25" ht="36" hidden="0" customHeight="1">
-      <x:c r="A25" s="16" t="str">
-        <x:v>Nine subjects outside the archived 76-subject cohort retain at least one trial in every class under the transparent 300 microvolt audit. No additional historical exclusion criterion is recorded for those nine subjects.</x:v>
-      </x:c>
-      <x:c r="B25" s="16"/>
-      <x:c r="C25" s="16"/>
-      <x:c r="D25" s="16"/>
-      <x:c r="E25" s="16"/>
-      <x:c r="F25" s="16"/>
-      <x:c r="G25" s="16"/>
-    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
     <x:mergeCell ref="A2:G2"/>
     <x:mergeCell ref="A23:G23"/>
     <x:mergeCell ref="A24:G24"/>
-    <x:mergeCell ref="A25:G25"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -653,7 +634,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>Archived 76-subject manuscript cohort with class-specific trial counts</x:v>
+        <x:v>Updated 85-subject cohort with at least one retained trial in every class</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1826,46 +1807,46 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="11" t="n">
-        <x:v>33</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="B28" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C28" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D28" s="11" t="n">
-        <x:v>88</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E28" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F28" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="G28" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H28" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="I28" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="J28" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K28" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="L28" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="M28" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N28" s="11" t="n">
-        <x:v>156</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="O28" s="11" t="str">
         <x:v>No</x:v>
@@ -1876,28 +1857,28 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="11" t="n">
-        <x:v>34</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B29" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C29" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D29" s="11" t="n">
-        <x:v>90</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="E29" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F29" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G29" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="H29" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I29" s="11" t="n">
         <x:v>0</x:v>
@@ -1912,10 +1893,10 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="M29" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="N29" s="11" t="n">
-        <x:v>154</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="O29" s="11" t="str">
         <x:v>No</x:v>
@@ -1926,7 +1907,7 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="11" t="n">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="B30" s="11" t="n">
         <x:v>90</x:v>
@@ -1938,25 +1919,25 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="E30" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F30" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G30" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H30" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="I30" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J30" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="K30" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="L30" s="11" t="n">
         <x:v>0</x:v>
@@ -1965,7 +1946,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="N30" s="11" t="n">
-        <x:v>156</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="O30" s="11" t="str">
         <x:v>No</x:v>
@@ -1976,46 +1957,46 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="11" t="n">
-        <x:v>36</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="B31" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C31" s="11" t="n">
-        <x:v>58</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D31" s="11" t="n">
-        <x:v>32</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E31" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F31" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G31" s="11" t="n">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="H31" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I31" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J31" s="11" t="n">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="K31" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="L31" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M31" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="N31" s="11" t="n">
-        <x:v>88</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="O31" s="11" t="str">
         <x:v>No</x:v>
@@ -2026,46 +2007,46 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="11" t="n">
-        <x:v>37</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B32" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C32" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D32" s="11" t="n">
-        <x:v>90</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E32" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="F32" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="G32" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="H32" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="I32" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J32" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="K32" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="L32" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M32" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="N32" s="11" t="n">
-        <x:v>154</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="O32" s="11" t="str">
         <x:v>No</x:v>
@@ -2076,146 +2057,146 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="11" t="n">
-        <x:v>38</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B33" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C33" s="11" t="n">
-        <x:v>11</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D33" s="11" t="n">
-        <x:v>79</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E33" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="F33" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G33" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="H33" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="I33" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J33" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="K33" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="L33" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M33" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="N33" s="11" t="n">
-        <x:v>142</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="O33" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="P33" s="11" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="11" t="n">
-        <x:v>40</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="B34" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C34" s="11" t="n">
-        <x:v>18</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D34" s="11" t="n">
-        <x:v>72</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="E34" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F34" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G34" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="H34" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="I34" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G34" s="11" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="H34" s="11" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="I34" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
       <x:c r="J34" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="K34" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="L34" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M34" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="N34" s="11" t="n">
-        <x:v>137</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="O34" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="P34" s="11" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="11" t="n">
-        <x:v>41</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B35" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C35" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="D35" s="11" t="n">
-        <x:v>90</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E35" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F35" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G35" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H35" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I35" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="J35" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="K35" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="L35" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="M35" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="N35" s="11" t="n">
-        <x:v>156</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="O35" s="11" t="str">
         <x:v>No</x:v>
@@ -2226,46 +2207,46 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="11" t="n">
-        <x:v>42</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B36" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C36" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D36" s="11" t="n">
-        <x:v>90</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E36" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F36" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G36" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="H36" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="I36" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J36" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="K36" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="L36" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M36" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="N36" s="11" t="n">
-        <x:v>156</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="O36" s="11" t="str">
         <x:v>No</x:v>
@@ -2276,46 +2257,46 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="11" t="n">
-        <x:v>44</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B37" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C37" s="11" t="n">
-        <x:v>82</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D37" s="11" t="n">
-        <x:v>8</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E37" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F37" s="11" t="n">
-        <x:v>18</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G37" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="H37" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="I37" s="11" t="n">
-        <x:v>18</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J37" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="K37" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="L37" s="11" t="n">
-        <x:v>15</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M37" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="N37" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="O37" s="11" t="str">
         <x:v>No</x:v>
@@ -2326,46 +2307,46 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="11" t="n">
-        <x:v>45</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B38" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C38" s="11" t="n">
-        <x:v>62</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D38" s="11" t="n">
-        <x:v>28</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E38" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F38" s="11" t="n">
-        <x:v>13</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G38" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="H38" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I38" s="11" t="n">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J38" s="11" t="n">
-        <x:v>14</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="K38" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="L38" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M38" s="11" t="n">
-        <x:v>9</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="N38" s="11" t="n">
-        <x:v>61</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="O38" s="11" t="str">
         <x:v>No</x:v>
@@ -2376,46 +2357,46 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="11" t="n">
-        <x:v>46</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B39" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C39" s="11" t="n">
-        <x:v>83</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D39" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E39" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F39" s="11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G39" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="H39" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="I39" s="11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J39" s="11" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="K39" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="L39" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="M39" s="11" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="E39" s="11" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="F39" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G39" s="11" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="H39" s="11" t="n">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="I39" s="11" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="J39" s="11" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K39" s="11" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="L39" s="11" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="M39" s="11" t="n">
-        <x:v>18</x:v>
-      </x:c>
       <x:c r="N39" s="11" t="n">
-        <x:v>65</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="O39" s="11" t="str">
         <x:v>No</x:v>
@@ -2426,46 +2407,46 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="11" t="n">
-        <x:v>47</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B40" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C40" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D40" s="11" t="n">
-        <x:v>90</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E40" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F40" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G40" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="H40" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I40" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="J40" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="K40" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="L40" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="M40" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="N40" s="11" t="n">
-        <x:v>157</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="O40" s="11" t="str">
         <x:v>No</x:v>
@@ -2476,46 +2457,46 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="11" t="n">
-        <x:v>50</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B41" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C41" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D41" s="11" t="n">
-        <x:v>90</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E41" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="F41" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G41" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="H41" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="I41" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J41" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="K41" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="L41" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M41" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="N41" s="11" t="n">
-        <x:v>156</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="O41" s="11" t="str">
         <x:v>No</x:v>
@@ -2526,7 +2507,7 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="11" t="n">
-        <x:v>51</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B42" s="11" t="n">
         <x:v>90</x:v>
@@ -2556,16 +2537,16 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="K42" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="L42" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M42" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="N42" s="11" t="n">
-        <x:v>159</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="O42" s="11" t="str">
         <x:v>No</x:v>
@@ -2576,46 +2557,46 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="11" t="n">
-        <x:v>52</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B43" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C43" s="11" t="n">
-        <x:v>80</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="D43" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E43" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F43" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G43" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H43" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="I43" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J43" s="11" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K43" s="11" t="n">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="F43" s="11" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="G43" s="11" t="n">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="H43" s="11" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="I43" s="11" t="n">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="J43" s="11" t="n">
+      <x:c r="L43" s="11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="M43" s="11" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="K43" s="11" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="L43" s="11" t="n">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="M43" s="11" t="n">
-        <x:v>11</x:v>
-      </x:c>
       <x:c r="N43" s="11" t="n">
-        <x:v>38</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="O43" s="11" t="str">
         <x:v>No</x:v>
@@ -2626,46 +2607,46 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="11" t="n">
-        <x:v>54</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B44" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C44" s="11" t="n">
-        <x:v>79</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D44" s="11" t="n">
-        <x:v>11</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E44" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="F44" s="11" t="n">
-        <x:v>15</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G44" s="11" t="n">
-        <x:v>8</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="H44" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="I44" s="11" t="n">
-        <x:v>14</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J44" s="11" t="n">
-        <x:v>8</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="K44" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="L44" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M44" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="N44" s="11" t="n">
-        <x:v>39</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="O44" s="11" t="str">
         <x:v>No</x:v>
@@ -2676,7 +2657,7 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="11" t="n">
-        <x:v>55</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="B45" s="11" t="n">
         <x:v>90</x:v>
@@ -2688,34 +2669,34 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="E45" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F45" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G45" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="H45" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="I45" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J45" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="K45" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="L45" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M45" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="N45" s="11" t="n">
-        <x:v>157</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="O45" s="11" t="str">
         <x:v>No</x:v>
@@ -2726,46 +2707,46 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="11" t="n">
-        <x:v>57</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B46" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C46" s="11" t="n">
-        <x:v>55</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D46" s="11" t="n">
-        <x:v>35</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="E46" s="11" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="F46" s="11" t="n">
-        <x:v>16</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="G46" s="11" t="n">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H46" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="I46" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="J46" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K46" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="L46" s="11" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J46" s="11" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="K46" s="11" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="L46" s="11" t="n">
+      <x:c r="M46" s="11" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="M46" s="11" t="n">
-        <x:v>12</x:v>
-      </x:c>
       <x:c r="N46" s="11" t="n">
-        <x:v>64</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="O46" s="11" t="str">
         <x:v>No</x:v>
@@ -2776,46 +2757,46 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="11" t="n">
-        <x:v>59</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B47" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C47" s="11" t="n">
-        <x:v>27</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D47" s="11" t="n">
-        <x:v>63</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="E47" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F47" s="11" t="n">
-        <x:v>9</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G47" s="11" t="n">
-        <x:v>15</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="H47" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I47" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="J47" s="11" t="n">
-        <x:v>14</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="K47" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="L47" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="M47" s="11" t="n">
-        <x:v>17</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="N47" s="11" t="n">
-        <x:v>109</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="O47" s="11" t="str">
         <x:v>No</x:v>
@@ -2826,7 +2807,7 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="11" t="n">
-        <x:v>62</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B48" s="11" t="n">
         <x:v>90</x:v>
@@ -2876,46 +2857,46 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="11" t="n">
-        <x:v>63</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B49" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C49" s="11" t="n">
-        <x:v>17</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D49" s="11" t="n">
-        <x:v>73</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E49" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="F49" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G49" s="11" t="n">
-        <x:v>17</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="H49" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="I49" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="J49" s="11" t="n">
-        <x:v>17</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="K49" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="L49" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="M49" s="11" t="n">
-        <x:v>18</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="N49" s="11" t="n">
-        <x:v>125</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="O49" s="11" t="str">
         <x:v>No</x:v>
@@ -2926,46 +2907,46 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="11" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B50" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C50" s="11" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="D50" s="11" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="E50" s="11" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F50" s="11" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G50" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="H50" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="I50" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="J50" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="K50" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="L50" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="M50" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="N50" s="11" t="n">
         <x:v>64</x:v>
-      </x:c>
-      <x:c r="B50" s="11" t="n">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="C50" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="D50" s="11" t="n">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="E50" s="11" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="F50" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G50" s="11" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="H50" s="11" t="n">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="I50" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J50" s="11" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="K50" s="11" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="L50" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M50" s="11" t="n">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="N50" s="11" t="n">
-        <x:v>156</x:v>
       </x:c>
       <x:c r="O50" s="11" t="str">
         <x:v>No</x:v>
@@ -2976,46 +2957,46 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="11" t="n">
-        <x:v>65</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="B51" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C51" s="11" t="n">
-        <x:v>55</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D51" s="11" t="n">
-        <x:v>35</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E51" s="11" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="F51" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="G51" s="11" t="n">
-        <x:v>19</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H51" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="I51" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="J51" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="K51" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="L51" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="M51" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J51" s="11" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="K51" s="11" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="L51" s="11" t="n">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="M51" s="11" t="n">
-        <x:v>17</x:v>
-      </x:c>
       <x:c r="N51" s="11" t="n">
-        <x:v>91</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="O51" s="11" t="str">
         <x:v>No</x:v>
@@ -3026,46 +3007,46 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="11" t="n">
-        <x:v>66</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B52" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C52" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D52" s="11" t="n">
-        <x:v>88</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E52" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F52" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G52" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H52" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="I52" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="J52" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="K52" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="L52" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="M52" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="N52" s="11" t="n">
-        <x:v>156</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="O52" s="11" t="str">
         <x:v>No</x:v>
@@ -3076,7 +3057,7 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="11" t="n">
-        <x:v>67</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B53" s="11" t="n">
         <x:v>90</x:v>
@@ -3088,22 +3069,22 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="E53" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F53" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G53" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="H53" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I53" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J53" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="K53" s="11" t="n">
         <x:v>22</x:v>
@@ -3126,46 +3107,46 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="11" t="n">
-        <x:v>68</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B54" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C54" s="11" t="n">
-        <x:v>45</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="D54" s="11" t="n">
-        <x:v>45</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="E54" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="F54" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G54" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H54" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="I54" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="J54" s="11" t="n">
-        <x:v>20</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="K54" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="L54" s="11" t="n">
-        <x:v>9</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="M54" s="11" t="n">
-        <x:v>14</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="N54" s="11" t="n">
-        <x:v>100</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="O54" s="11" t="str">
         <x:v>No</x:v>
@@ -3176,46 +3157,46 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="11" t="n">
-        <x:v>69</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B55" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C55" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D55" s="11" t="n">
-        <x:v>69</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E55" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F55" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G55" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="H55" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I55" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J55" s="11" t="n">
-        <x:v>19</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="K55" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="L55" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M55" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="N55" s="11" t="n">
-        <x:v>133</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="O55" s="11" t="str">
         <x:v>No</x:v>
@@ -3226,46 +3207,46 @@
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="11" t="n">
-        <x:v>70</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B56" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C56" s="11" t="n">
-        <x:v>26</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D56" s="11" t="n">
-        <x:v>64</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E56" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F56" s="11" t="n">
-        <x:v>11</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G56" s="11" t="n">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="H56" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="I56" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J56" s="11" t="n">
-        <x:v>11</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="K56" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="L56" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="M56" s="11" t="n">
-        <x:v>20</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="N56" s="11" t="n">
-        <x:v>106</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="O56" s="11" t="str">
         <x:v>No</x:v>
@@ -3276,46 +3257,46 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="11" t="n">
-        <x:v>71</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B57" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C57" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D57" s="11" t="n">
-        <x:v>69</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="E57" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="F57" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G57" s="11" t="n">
-        <x:v>17</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="H57" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="I57" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J57" s="11" t="n">
-        <x:v>16</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="K57" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="L57" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M57" s="11" t="n">
-        <x:v>18</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="N57" s="11" t="n">
-        <x:v>120</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="O57" s="11" t="str">
         <x:v>No</x:v>
@@ -3326,7 +3307,7 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="11" t="n">
-        <x:v>72</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B58" s="11" t="n">
         <x:v>90</x:v>
@@ -3353,19 +3334,19 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J58" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="K58" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="L58" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M58" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="N58" s="11" t="n">
-        <x:v>154</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="O58" s="11" t="str">
         <x:v>No</x:v>
@@ -3376,96 +3357,96 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="11" t="n">
-        <x:v>73</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B59" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C59" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D59" s="11" t="n">
-        <x:v>90</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="E59" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F59" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G59" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="H59" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I59" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J59" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="K59" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="L59" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="M59" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="N59" s="11" t="n">
-        <x:v>153</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="O59" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="P59" s="11" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="11" t="n">
-        <x:v>74</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B60" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C60" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D60" s="11" t="n">
-        <x:v>90</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E60" s="11" t="n">
         <x:v>24</x:v>
       </x:c>
       <x:c r="F60" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G60" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="H60" s="11" t="n">
         <x:v>21</x:v>
       </x:c>
       <x:c r="I60" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J60" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="K60" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="L60" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M60" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="N60" s="11" t="n">
-        <x:v>154</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="O60" s="11" t="str">
         <x:v>No</x:v>
@@ -3476,146 +3457,146 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="11" t="n">
-        <x:v>75</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B61" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C61" s="11" t="n">
-        <x:v>83</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D61" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E61" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="F61" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="G61" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H61" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="I61" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="J61" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="K61" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="L61" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M61" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="N61" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="O61" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="P61" s="11" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="11" t="n">
-        <x:v>76</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B62" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C62" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="D62" s="11" t="n">
-        <x:v>90</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E62" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F62" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G62" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="H62" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I62" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="J62" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="K62" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="L62" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="M62" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="N62" s="11" t="n">
-        <x:v>153</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="O62" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="P62" s="11" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="11" t="n">
-        <x:v>77</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="B63" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C63" s="11" t="n">
-        <x:v>59</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D63" s="11" t="n">
-        <x:v>31</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E63" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F63" s="11" t="n">
-        <x:v>9</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G63" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="H63" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I63" s="11" t="n">
-        <x:v>14</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J63" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="K63" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="L63" s="11" t="n">
-        <x:v>17</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M63" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="N63" s="11" t="n">
-        <x:v>59</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="O63" s="11" t="str">
         <x:v>No</x:v>
@@ -3626,7 +3607,7 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="11" t="n">
-        <x:v>78</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B64" s="11" t="n">
         <x:v>90</x:v>
@@ -3644,7 +3625,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G64" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H64" s="11" t="n">
         <x:v>22</x:v>
@@ -3653,69 +3634,69 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="J64" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="K64" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="L64" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M64" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="N64" s="11" t="n">
-        <x:v>158</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="O64" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="P64" s="11" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="11" t="n">
-        <x:v>79</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B65" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C65" s="11" t="n">
-        <x:v>63</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D65" s="11" t="n">
-        <x:v>27</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E65" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="F65" s="11" t="n">
-        <x:v>18</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G65" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="H65" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="I65" s="11" t="n">
-        <x:v>20</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J65" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="K65" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="L65" s="11" t="n">
-        <x:v>13</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M65" s="11" t="n">
-        <x:v>11</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="N65" s="11" t="n">
-        <x:v>45</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="O65" s="11" t="str">
         <x:v>No</x:v>
@@ -3726,57 +3707,57 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="11" t="n">
-        <x:v>80</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="B66" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C66" s="11" t="n">
-        <x:v>62</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="D66" s="11" t="n">
-        <x:v>28</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E66" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F66" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="G66" s="11" t="n">
-        <x:v>20</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H66" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I66" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="J66" s="11" t="n">
-        <x:v>17</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="K66" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="L66" s="11" t="n">
-        <x:v>9</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="M66" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="N66" s="11" t="n">
-        <x:v>77</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="O66" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="P66" s="11" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="11" t="n">
-        <x:v>81</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B67" s="11" t="n">
         <x:v>90</x:v>
@@ -3788,84 +3769,84 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="E67" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F67" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G67" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H67" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I67" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J67" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="K67" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="L67" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M67" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="N67" s="11" t="n">
-        <x:v>158</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="O67" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="P67" s="11" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="11" t="n">
-        <x:v>82</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B68" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C68" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="D68" s="11" t="n">
-        <x:v>89</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E68" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F68" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G68" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="H68" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="I68" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="J68" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="K68" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="L68" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="M68" s="11" t="n">
-        <x:v>20</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="N68" s="11" t="n">
-        <x:v>152</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="O68" s="11" t="str">
         <x:v>No</x:v>
@@ -3876,96 +3857,96 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="11" t="n">
-        <x:v>84</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="B69" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C69" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D69" s="11" t="n">
-        <x:v>83</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E69" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="F69" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G69" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="H69" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="I69" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J69" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="K69" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="L69" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M69" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="N69" s="11" t="n">
-        <x:v>146</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="O69" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="P69" s="11" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="11" t="n">
-        <x:v>85</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B70" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C70" s="11" t="n">
-        <x:v>19</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D70" s="11" t="n">
-        <x:v>71</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E70" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F70" s="11" t="n">
-        <x:v>5</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G70" s="11" t="n">
-        <x:v>18</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H70" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I70" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="J70" s="11" t="n">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="K70" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="L70" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="M70" s="11" t="n">
-        <x:v>19</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="N70" s="11" t="n">
-        <x:v>123</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="O70" s="11" t="str">
         <x:v>No</x:v>
@@ -3976,46 +3957,46 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="11" t="n">
-        <x:v>87</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B71" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C71" s="11" t="n">
-        <x:v>29</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D71" s="11" t="n">
-        <x:v>61</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E71" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F71" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G71" s="11" t="n">
-        <x:v>15</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="H71" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I71" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J71" s="11" t="n">
-        <x:v>20</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="K71" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="L71" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="M71" s="11" t="n">
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="N71" s="11" t="n">
-        <x:v>111</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="O71" s="11" t="str">
         <x:v>No</x:v>
@@ -4026,46 +4007,46 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="11" t="n">
-        <x:v>93</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B72" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C72" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D72" s="11" t="n">
-        <x:v>89</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="E72" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F72" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G72" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="H72" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I72" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J72" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="K72" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="L72" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="M72" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="N72" s="11" t="n">
-        <x:v>156</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="O72" s="11" t="str">
         <x:v>No</x:v>
@@ -4076,46 +4057,46 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="11" t="n">
-        <x:v>94</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="B73" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C73" s="11" t="n">
-        <x:v>77</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D73" s="11" t="n">
-        <x:v>13</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="E73" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F73" s="11" t="n">
-        <x:v>13</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G73" s="11" t="n">
-        <x:v>9</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="H73" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I73" s="11" t="n">
-        <x:v>9</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J73" s="11" t="n">
-        <x:v>14</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="K73" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="L73" s="11" t="n">
-        <x:v>11</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M73" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="N73" s="11" t="n">
-        <x:v>48</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="O73" s="11" t="str">
         <x:v>No</x:v>
@@ -4126,46 +4107,46 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="11" t="n">
-        <x:v>95</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B74" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C74" s="11" t="n">
-        <x:v>71</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D74" s="11" t="n">
-        <x:v>19</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E74" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F74" s="11" t="n">
-        <x:v>16</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G74" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H74" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="I74" s="11" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="J74" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="K74" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="L74" s="11" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="M74" s="11" t="n">
-        <x:v>8</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="N74" s="11" t="n">
-        <x:v>40</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="O74" s="11" t="str">
         <x:v>No</x:v>
@@ -4176,96 +4157,96 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="11" t="n">
-        <x:v>98</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="B75" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C75" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D75" s="11" t="n">
-        <x:v>90</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="E75" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="F75" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G75" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="H75" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="I75" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J75" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="K75" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="L75" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M75" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="N75" s="11" t="n">
-        <x:v>159</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="O75" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="P75" s="11" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="11" t="n">
-        <x:v>101</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="B76" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C76" s="11" t="n">
-        <x:v>30</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D76" s="11" t="n">
-        <x:v>60</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E76" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F76" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G76" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="H76" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I76" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="J76" s="11" t="n">
-        <x:v>23</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="K76" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="L76" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="M76" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="N76" s="11" t="n">
-        <x:v>126</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="O76" s="11" t="str">
         <x:v>No</x:v>
@@ -4276,46 +4257,46 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="11" t="n">
-        <x:v>102</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B77" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C77" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="D77" s="11" t="n">
-        <x:v>90</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E77" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="F77" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G77" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H77" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="I77" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="J77" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="K77" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="L77" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="M77" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="N77" s="11" t="n">
-        <x:v>154</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="O77" s="11" t="str">
         <x:v>No</x:v>
@@ -4326,46 +4307,46 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="11" t="n">
-        <x:v>103</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B78" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C78" s="11" t="n">
-        <x:v>59</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D78" s="11" t="n">
-        <x:v>31</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="E78" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="F78" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="G78" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="H78" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="I78" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="J78" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="K78" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="L78" s="11" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="J78" s="11" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="K78" s="11" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="L78" s="11" t="n">
+      <x:c r="M78" s="11" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="M78" s="11" t="n">
-        <x:v>8</x:v>
-      </x:c>
       <x:c r="N78" s="11" t="n">
-        <x:v>67</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="O78" s="11" t="str">
         <x:v>No</x:v>
@@ -4376,46 +4357,46 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="11" t="n">
-        <x:v>105</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="B79" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C79" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D79" s="11" t="n">
-        <x:v>87</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="E79" s="11" t="n">
         <x:v>23</x:v>
       </x:c>
       <x:c r="F79" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G79" s="11" t="n">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="H79" s="11" t="n">
         <x:v>22</x:v>
       </x:c>
       <x:c r="I79" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="J79" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="K79" s="11" t="n">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="L79" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="M79" s="11" t="n">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="N79" s="11" t="n">
-        <x:v>150</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="O79" s="11" t="str">
         <x:v>No</x:v>
@@ -4426,46 +4407,46 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="11" t="n">
-        <x:v>106</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B80" s="11" t="n">
         <x:v>90</x:v>
       </x:c>
       <x:c r="C80" s="11" t="n">
-        <x:v>70</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D80" s="11" t="n">
-        <x:v>20</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E80" s="11" t="n">
-        <x:v>24</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F80" s="11" t="n">
         <x:v>13</x:v>
       </x:c>
       <x:c r="G80" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="H80" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="I80" s="11" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="J80" s="11" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="K80" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="L80" s="11" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="H80" s="11" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="I80" s="11" t="n">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="J80" s="11" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="K80" s="11" t="n">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="L80" s="11" t="n">
-        <x:v>16</x:v>
-      </x:c>
       <x:c r="M80" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="N80" s="11" t="n">
-        <x:v>45</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="O80" s="11" t="str">
         <x:v>No</x:v>
@@ -4476,51 +4457,501 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="11" t="n">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="B81" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C81" s="11" t="n">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="D81" s="11" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="E81" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F81" s="11" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G81" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H81" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="I81" s="11" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="J81" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="K81" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="L81" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="M81" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N81" s="11" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="O81" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P81" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82">
+      <x:c r="A82" s="11" t="n">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="B82" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C82" s="11" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="D82" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E82" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F82" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G82" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H82" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="I82" s="11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="J82" s="11" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="K82" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="L82" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="M82" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="N82" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="O82" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P82" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" s="11" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B83" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C83" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D83" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E83" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F83" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G83" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="H83" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="I83" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J83" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="K83" s="11" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="L83" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M83" s="11" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="N83" s="11" t="n">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="O83" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P83" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84">
+      <x:c r="A84" s="11" t="n">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="B84" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C84" s="11" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D84" s="11" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="E84" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F84" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="G84" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H84" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="I84" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J84" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K84" s="11" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="L84" s="11" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="M84" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N84" s="11" t="n">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="O84" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P84" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="11" t="n">
+        <x:v>101</x:v>
+      </x:c>
+      <x:c r="B85" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C85" s="11" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D85" s="11" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="E85" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F85" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G85" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H85" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="I85" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J85" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="K85" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="L85" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M85" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="N85" s="11" t="n">
+        <x:v>126</x:v>
+      </x:c>
+      <x:c r="O85" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P85" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="11" t="n">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B86" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C86" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D86" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="E86" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F86" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G86" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="H86" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="I86" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J86" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="K86" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="L86" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M86" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="N86" s="11" t="n">
+        <x:v>154</x:v>
+      </x:c>
+      <x:c r="O86" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P86" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="11" t="n">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="B87" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C87" s="11" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="D87" s="11" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E87" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F87" s="11" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="G87" s="11" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="H87" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="I87" s="11" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="J87" s="11" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="K87" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="L87" s="11" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="M87" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="N87" s="11" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="O87" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P87" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="11" t="n">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="B88" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C88" s="11" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D88" s="11" t="n">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="E88" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F88" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G88" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="H88" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="I88" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J88" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="K88" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="L88" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="M88" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="N88" s="11" t="n">
+        <x:v>150</x:v>
+      </x:c>
+      <x:c r="O88" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P88" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="11" t="n">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="B89" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C89" s="11" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="D89" s="11" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E89" s="11" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F89" s="11" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="G89" s="11" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H89" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="I89" s="11" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="J89" s="11" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="K89" s="11" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="L89" s="11" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="M89" s="11" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="N89" s="11" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="O89" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P89" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="11" t="n">
         <x:v>107</x:v>
       </x:c>
-      <x:c r="B81" s="11" t="n">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="C81" s="11" t="n">
+      <x:c r="B90" s="11" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C90" s="11" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="D81" s="11" t="n">
+      <x:c r="D90" s="11" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="E81" s="11" t="n">
+      <x:c r="E90" s="11" t="n">
         <x:v>24</x:v>
       </x:c>
-      <x:c r="F81" s="11" t="n">
+      <x:c r="F90" s="11" t="n">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="G81" s="11" t="n">
+      <x:c r="G90" s="11" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="H81" s="11" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="I81" s="11" t="n">
+      <x:c r="H90" s="11" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="I90" s="11" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="J81" s="11" t="n">
+      <x:c r="J90" s="11" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="K81" s="11" t="n">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="L81" s="11" t="n">
+      <x:c r="K90" s="11" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="L90" s="11" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="M81" s="11" t="n">
+      <x:c r="M90" s="11" t="n">
         <x:v>14</x:v>
       </x:c>
-      <x:c r="N81" s="11" t="n">
+      <x:c r="N90" s="11" t="n">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="O81" s="11" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P81" s="11" t="str">
+      <x:c r="O90" s="11" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P90" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
     </x:row>
@@ -4549,12 +4980,12 @@
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
       <x:c r="A1" s="1" t="str">
-        <x:v>Subjects outside the manuscript physiology cohort</x:v>
+        <x:v>Subjects excluded from physiology analysis</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>Twenty-seven classification-eligible subjects not included in the archived 76-subject physiology cohort</x:v>
+        <x:v>Eighteen subjects with no retained trials in at least one class under the 300 microvolt rule</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -4829,59 +5260,59 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="11" t="n">
-        <x:v>32</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B15" s="17" t="str">
-        <x:v>Not selected in archived 76-subject cohort; additional historical criterion not recorded</x:v>
+        <x:v>all rest trials exceeded 300uv</x:v>
       </x:c>
       <x:c r="C15" s="11" t="str">
-        <x:v>Not recorded</x:v>
+        <x:v>Rest</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="E15" s="11" t="n">
-        <x:v>13</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F15" s="11" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G15" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G15" s="11" t="n">
-        <x:v>4</x:v>
-      </x:c>
       <x:c r="H15" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="11" t="n">
-        <x:v>39</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B16" s="17" t="str">
-        <x:v>Not selected in archived 76-subject cohort; additional historical criterion not recorded</x:v>
+        <x:v>all rest trials exceeded 300uv</x:v>
       </x:c>
       <x:c r="C16" s="11" t="str">
-        <x:v>Not recorded</x:v>
+        <x:v>Rest</x:v>
       </x:c>
       <x:c r="D16" s="11" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="E16" s="11" t="n">
-        <x:v>25</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F16" s="11" t="n">
-        <x:v>7</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G16" s="11" t="n">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H16" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="11" t="n">
-        <x:v>48</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B17" s="17" t="str">
         <x:v>all rest trials exceeded 300uv</x:v>
@@ -4902,38 +5333,38 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="H17" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="11" t="n">
-        <x:v>49</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B18" s="17" t="str">
-        <x:v>Not selected in archived 76-subject cohort; additional historical criterion not recorded</x:v>
+        <x:v>all rest trials exceeded 300uv</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
-        <x:v>Not recorded</x:v>
+        <x:v>Rest</x:v>
       </x:c>
       <x:c r="D18" s="11" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="E18" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F18" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G18" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H18" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="11" t="n">
-        <x:v>53</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B19" s="17" t="str">
         <x:v>all rest trials exceeded 300uv</x:v>
@@ -4948,96 +5379,96 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F19" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G19" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H19" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="11" t="n">
-        <x:v>56</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B20" s="17" t="str">
-        <x:v>Not selected in archived 76-subject cohort; additional historical criterion not recorded</x:v>
+        <x:v>all rest trials exceeded 300uv</x:v>
       </x:c>
       <x:c r="C20" s="11" t="str">
-        <x:v>Not recorded</x:v>
+        <x:v>Rest</x:v>
       </x:c>
       <x:c r="D20" s="11" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="E20" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F20" s="11" t="n">
-        <x:v>6</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G20" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H20" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="11" t="n">
-        <x:v>58</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="B21" s="17" t="str">
-        <x:v>Not selected in archived 76-subject cohort; additional historical criterion not recorded</x:v>
+        <x:v>all rest trials exceeded 300uv</x:v>
       </x:c>
       <x:c r="C21" s="11" t="str">
-        <x:v>Not recorded</x:v>
+        <x:v>Rest</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="E21" s="11" t="n">
-        <x:v>27</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F21" s="11" t="n">
-        <x:v>12</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="G21" s="11" t="n">
-        <x:v>10</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H21" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="11" t="n">
-        <x:v>60</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B22" s="17" t="str">
-        <x:v>all rest trials exceeded 300uv</x:v>
+        <x:v>all right fist imagery trials exceeded 300uv</x:v>
       </x:c>
       <x:c r="C22" s="11" t="str">
-        <x:v>Rest</x:v>
+        <x:v>Right fist imagery</x:v>
       </x:c>
       <x:c r="D22" s="11" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="E22" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F22" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G22" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H22" s="11" t="n">
-        <x:v>0</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="11" t="n">
-        <x:v>61</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B23" s="17" t="str">
         <x:v>all rest trials exceeded 300uv</x:v>
@@ -5055,243 +5486,9 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="G23" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H23" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
-      <x:c r="A24" s="11" t="n">
-        <x:v>83</x:v>
-      </x:c>
-      <x:c r="B24" s="17" t="str">
-        <x:v>Not selected in archived 76-subject cohort; additional historical criterion not recorded</x:v>
-      </x:c>
-      <x:c r="C24" s="11" t="str">
-        <x:v>Not recorded</x:v>
-      </x:c>
-      <x:c r="D24" s="11" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="E24" s="11" t="n">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F24" s="11" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G24" s="11" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="H24" s="11" t="n">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="15" hidden="0" customHeight="1">
-      <x:c r="A25" s="11" t="n">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="B25" s="17" t="str">
-        <x:v>Not selected in archived 76-subject cohort; additional historical criterion not recorded</x:v>
-      </x:c>
-      <x:c r="C25" s="11" t="str">
-        <x:v>Not recorded</x:v>
-      </x:c>
-      <x:c r="D25" s="11" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="E25" s="11" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F25" s="11" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="G25" s="11" t="n">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="H25" s="11" t="n">
-        <x:v>22</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="15" hidden="0" customHeight="1">
-      <x:c r="A26" s="11" t="n">
-        <x:v>90</x:v>
-      </x:c>
-      <x:c r="B26" s="17" t="str">
-        <x:v>all rest trials exceeded 300uv</x:v>
-      </x:c>
-      <x:c r="C26" s="11" t="str">
-        <x:v>Rest</x:v>
-      </x:c>
-      <x:c r="D26" s="11" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E26" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F26" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G26" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H26" s="11" t="n">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="15" hidden="0" customHeight="1">
-      <x:c r="A27" s="11" t="n">
-        <x:v>91</x:v>
-      </x:c>
-      <x:c r="B27" s="17" t="str">
-        <x:v>all rest trials exceeded 300uv</x:v>
-      </x:c>
-      <x:c r="C27" s="11" t="str">
-        <x:v>Rest</x:v>
-      </x:c>
-      <x:c r="D27" s="11" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E27" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F27" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G27" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H27" s="11" t="n">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="15" hidden="0" customHeight="1">
-      <x:c r="A28" s="11" t="n">
-        <x:v>96</x:v>
-      </x:c>
-      <x:c r="B28" s="17" t="str">
-        <x:v>all rest trials exceeded 300uv</x:v>
-      </x:c>
-      <x:c r="C28" s="11" t="str">
-        <x:v>Rest</x:v>
-      </x:c>
-      <x:c r="D28" s="11" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E28" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F28" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G28" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H28" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="15" hidden="0" customHeight="1">
-      <x:c r="A29" s="11" t="n">
-        <x:v>97</x:v>
-      </x:c>
-      <x:c r="B29" s="17" t="str">
-        <x:v>Not selected in archived 76-subject cohort; additional historical criterion not recorded</x:v>
-      </x:c>
-      <x:c r="C29" s="11" t="str">
-        <x:v>Not recorded</x:v>
-      </x:c>
-      <x:c r="D29" s="11" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="E29" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="F29" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G29" s="11" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H29" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="15" hidden="0" customHeight="1">
-      <x:c r="A30" s="11" t="n">
-        <x:v>99</x:v>
-      </x:c>
-      <x:c r="B30" s="17" t="str">
-        <x:v>Not selected in archived 76-subject cohort; additional historical criterion not recorded</x:v>
-      </x:c>
-      <x:c r="C30" s="11" t="str">
-        <x:v>Not recorded</x:v>
-      </x:c>
-      <x:c r="D30" s="11" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="E30" s="11" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="F30" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G30" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="H30" s="11" t="n">
-        <x:v>6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="15" hidden="0" customHeight="1">
-      <x:c r="A31" s="11" t="n">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="B31" s="17" t="str">
-        <x:v>all right fist imagery trials exceeded 300uv</x:v>
-      </x:c>
-      <x:c r="C31" s="11" t="str">
-        <x:v>Right fist imagery</x:v>
-      </x:c>
-      <x:c r="D31" s="11" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E31" s="11" t="n">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="F31" s="11" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G31" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H31" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="15" hidden="0" customHeight="1">
-      <x:c r="A32" s="11" t="n">
-        <x:v>109</x:v>
-      </x:c>
-      <x:c r="B32" s="17" t="str">
-        <x:v>all rest trials exceeded 300uv</x:v>
-      </x:c>
-      <x:c r="C32" s="11" t="str">
-        <x:v>Rest</x:v>
-      </x:c>
-      <x:c r="D32" s="11" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="E32" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F32" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G32" s="11" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H32" s="11" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -5366,10 +5563,10 @@
         <x:v>Physiology cohort</x:v>
       </x:c>
       <x:c r="B8" s="17" t="str">
-        <x:v>76 subjects listed in Included Subjects</x:v>
+        <x:v>85 subjects listed in Included Subjects</x:v>
       </x:c>
       <x:c r="C8" s="17" t="str">
-        <x:v>Archived signal_analysis_summary.json</x:v>
+        <x:v>Updated signal_analysis_summary.json</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">

</xml_diff>